<commit_message>
Add wealth product analysis demo
</commit_message>
<xml_diff>
--- a/shared-templates/team_skill_register.xlsx
+++ b/shared-templates/team_skill_register.xlsx
@@ -2933,17 +2933,17 @@
       </c>
       <c r="K6" s="24" t="inlineStr">
         <is>
-          <t>产品解读、行业配置变化、净值走势、客户沟通要点</t>
+          <t>产品解读、净值归因、风险提示、客户沟通话术</t>
         </is>
       </c>
       <c r="L6" s="24" t="inlineStr">
         <is>
-          <t>规划</t>
+          <t>已制作Demo</t>
         </is>
       </c>
       <c r="M6" s="24" t="inlineStr">
         <is>
-          <t>catalog</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="N6" s="24" t="inlineStr">
@@ -2958,26 +2958,30 @@
       </c>
       <c r="P6" s="24" t="inlineStr">
         <is>
-          <t>保留为平台中立目录项；真实演示可复用 Dumate 能力，网页侧补一个轻量 Demo。</t>
-        </is>
-      </c>
-      <c r="Q6" s="24" t="str"/>
-      <c r="R6" s="24" t="str"/>
-      <c r="S6" s="24" t="str"/>
-      <c r="T6" s="24" t="str"/>
+          <t>已接入同事提供的页面 Demo；暂无真实 SKILL.md 与配套脚本，后续需补 Skill 包后再进入真实文件展示。</t>
+        </is>
+      </c>
+      <c r="Q6" s="24" t="inlineStr"/>
+      <c r="R6" s="24" t="inlineStr">
+        <is>
+          <t>presales-skill-matrix/wealth-product-net-value-analysis/wealth-product-net-value-analysis-demo.html</t>
+        </is>
+      </c>
+      <c r="S6" s="24" t="inlineStr"/>
+      <c r="T6" s="24" t="inlineStr"/>
       <c r="U6" s="24" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.2.0-demo</t>
         </is>
       </c>
       <c r="V6" s="24" t="inlineStr">
         <is>
-          <t>财富管理,投顾,产品解读,金融数据</t>
+          <t>财富管理,投顾,产品解读,净值走势,客户沟通,Demo</t>
         </is>
       </c>
       <c r="W6" s="24" t="inlineStr">
         <is>
-          <t>来源：Dumate场景积累-2026.05.29.pdf；仅先登记名称和分类，待补 SKILL.md。</t>
+          <t>2026-06-18 接入同事提供的财富产品解读与净值走势分析页面 Demo；当前仅有 HTML demo 文件，未伪造 Skill 文件包。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fund advisor skill package
</commit_message>
<xml_diff>
--- a/shared-templates/team_skill_register.xlsx
+++ b/shared-templates/team_skill_register.xlsx
@@ -2918,7 +2918,7 @@
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>面向投顾、理财经理、客户经理，在财富营销和陪伴过程中解读基金、股票、债券等产品，并支持持仓变化和净值走势分析。</t>
+          <t>面向投顾、理财经理、客户经理，围绕基金/财富产品进行材料解读、净值走势分析、持仓识别、量化评估和客户沟通话术生成。</t>
         </is>
       </c>
       <c r="I6" s="24" t="inlineStr">
@@ -2928,17 +2928,17 @@
       </c>
       <c r="J6" s="24" t="inlineStr">
         <is>
-          <t>产品材料、持仓截图、净值数据、客户问题</t>
+          <t>产品材料、持仓截图、净值数据、客户问题、基金/经理/公司数据</t>
         </is>
       </c>
       <c r="K6" s="24" t="inlineStr">
         <is>
-          <t>产品解读、净值归因、风险提示、客户沟通话术</t>
+          <t>产品解读、净值归因、量化分析、风险提示、客户沟通话术、持仓报告</t>
         </is>
       </c>
       <c r="L6" s="24" t="inlineStr">
         <is>
-          <t>已制作Demo</t>
+          <t>已开发</t>
         </is>
       </c>
       <c r="M6" s="24" t="inlineStr">
@@ -2948,40 +2948,52 @@
       </c>
       <c r="N6" s="24" t="inlineStr">
         <is>
-          <t>同事/Dumate场景积累</t>
+          <t>同事/Fund Advisor Skill包</t>
         </is>
       </c>
       <c r="O6" s="24" t="inlineStr">
         <is>
-          <t>Dumate</t>
+          <t>Dumate/Dodo</t>
         </is>
       </c>
       <c r="P6" s="24" t="inlineStr">
         <is>
-          <t>已接入同事提供的页面 Demo；暂无真实 SKILL.md 与配套脚本，后续需补 Skill 包后再进入真实文件展示。</t>
-        </is>
-      </c>
-      <c r="Q6" s="24" t="inlineStr"/>
+          <t>已补齐 fund-advisor 真实 Skill 包；页面 Demo 与真实 SKILL.md、脚本、数据、引用文档共同展示。后续可继续做 Web UI 运行验证和真实数据接入。</t>
+        </is>
+      </c>
+      <c r="Q6" s="24" t="inlineStr">
+        <is>
+          <t>presales-skill-matrix/wealth-product-net-value-analysis/SKILL.md</t>
+        </is>
+      </c>
       <c r="R6" s="24" t="inlineStr">
         <is>
           <t>presales-skill-matrix/wealth-product-net-value-analysis/wealth-product-net-value-analysis-demo.html</t>
         </is>
       </c>
-      <c r="S6" s="24" t="inlineStr"/>
-      <c r="T6" s="24" t="inlineStr"/>
+      <c r="S6" s="24" t="inlineStr">
+        <is>
+          <t>presales-skill-matrix/wealth-product-net-value-analysis/references/</t>
+        </is>
+      </c>
+      <c r="T6" s="24" t="inlineStr">
+        <is>
+          <t>presales-skill-matrix/wealth-product-net-value-analysis/data/</t>
+        </is>
+      </c>
       <c r="U6" s="24" t="inlineStr">
         <is>
-          <t>0.2.0-demo</t>
+          <t>5.0.0</t>
         </is>
       </c>
       <c r="V6" s="24" t="inlineStr">
         <is>
-          <t>财富管理,投顾,产品解读,净值走势,客户沟通,Demo</t>
+          <t>财富管理,基金投顾,产品解读,净值走势,持仓识别,量化分析,客户沟通,已开发Skill</t>
         </is>
       </c>
       <c r="W6" s="24" t="inlineStr">
         <is>
-          <t>2026-06-18 接入同事提供的财富产品解读与净值走势分析页面 Demo；当前仅有 HTML demo 文件，未伪造 Skill 文件包。</t>
+          <t>2026-06-18 已接入 fund-advisor 完整 Skill 包；保留同事提供的财富产品解读页面 Demo。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align credit due diligence demo with real skill package
</commit_message>
<xml_diff>
--- a/shared-templates/team_skill_register.xlsx
+++ b/shared-templates/team_skill_register.xlsx
@@ -8,9 +8,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已制作Skill登记" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="同事填写说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'已制作Skill登记'!$A$1:$AA$220</definedName>
-  </definedNames>
+  <definedNames/>
 </workbook>
 </file>
 
@@ -189,16 +187,16 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="004C1D95"/>
+      <color rgb="FF4C1D95"/>
     </font>
   </fonts>
   <fills count="41">
@@ -385,22 +383,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004C1D95"/>
+        <fgColor rgb="FF4C1D95"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006D28D9"/>
+        <fgColor rgb="FF6D28D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00334155"/>
+        <fgColor rgb="FF334155"/>
       </patternFill>
     </fill>
   </fills>
@@ -501,62 +499,62 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="FFD9E2F3"/>
       </left>
       <right style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="FFD9E2F3"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="FFD9E2F3"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="FFD9E2F3"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </left>
       <right style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </bottom>
     </border>
     <border>
       <top style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </top>
     </border>
     <border>
       <right style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </top>
     </border>
     <border>
       <top style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </bottom>
     </border>
     <border>
       <right style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2EC"/>
+        <color rgb="FFD9E2EC"/>
       </bottom>
     </border>
   </borders>
@@ -1166,9 +1164,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2571,17 +2569,17 @@
       </c>
       <c r="C6" s="37" t="inlineStr">
         <is>
-          <t>风控 / 财富管理 / 投研 / 团队管理 / 投标 / 方案写作 / 技术评估 / 资料检索 / 合规 / 车险 / 客服 / 办公 / 科技</t>
+          <t>AI信贷 / 信贷 / 贷前 / 贷中 / 贷后 / 风控 / 财富管理 / 投研 / 营销 / 客服 / 合规 / 团队管理 / 投标 / 方案写作 / 技术评估 / 资料检索 / 车险 / 办公 / 科技</t>
         </is>
       </c>
       <c r="D6" s="37" t="inlineStr">
         <is>
-          <t>用业务语言，不用技术语言。不要填“混合型”“Agent”“RAG”；这些属于实现模式。</t>
+          <t>用业务语言，不用技术语言。业务分类填最主要的业务入口；如果一个场景可被多个入口命中，在标签中补充相关业务词。面向客户专项演示时，可使用 AI信贷 这类演示集合标签。不要填“混合型”“Agent”“RAG”；这些属于实现模式。</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
         <is>
-          <t>授信走访=风控；个股研究=投研；日报汇总=团队管理；招标红线=投标</t>
+          <t>信贷尽调=业务分类填信贷，标签补 AI信贷、风控、贷前、尽调；授信走访=AI信贷/风控/信贷；贷后监测=AI信贷/贷后/风控</t>
         </is>
       </c>
     </row>
@@ -2778,8 +2776,16 @@
       <c r="A14" s="37" t="inlineStr"/>
       <c r="B14" s="37" t="inlineStr"/>
       <c r="C14" s="37" t="inlineStr"/>
-      <c r="D14" s="37" t="inlineStr"/>
-      <c r="E14" s="37" t="inlineStr"/>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>放不适合作为稳定主分类的关键词、产品名、平台名、项目名、指标名，也可补充辅助筛选的业务词或演示集合标签。</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>AI信贷,信贷,风控,贷前,尽调,P800,净值走势,日报,信创,投顾</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1" s="29">
       <c r="A15" s="37" t="inlineStr">
@@ -2861,7 +2867,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B2:E2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -5495,33 +5501,129 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="n"/>
-      <c r="B22" s="24" t="n"/>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24" t="n"/>
-      <c r="I22" s="24" t="n"/>
-      <c r="J22" s="24" t="n"/>
-      <c r="K22" s="24" t="n"/>
-      <c r="L22" s="24" t="n"/>
-      <c r="M22" s="24" t="n"/>
-      <c r="N22" s="24" t="n"/>
-      <c r="O22" s="24" t="n"/>
-      <c r="P22" s="24" t="n"/>
-      <c r="Q22" s="24" t="n"/>
-      <c r="R22" s="24" t="n"/>
-      <c r="S22" s="24" t="n"/>
-      <c r="T22" s="24" t="n"/>
-      <c r="U22" s="24" t="n"/>
-      <c r="V22" s="24" t="n"/>
-      <c r="W22" s="24" t="n"/>
-      <c r="X22" s="24" t="n"/>
-      <c r="Y22" s="24" t="n"/>
-      <c r="Z22" s="24" t="n"/>
-      <c r="AA22" s="24" t="n"/>
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>credit-due-diligence-report</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>信贷尽调调查与分析报告生成</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>客户金融场景</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>银行</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>中台</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>信贷</t>
+        </is>
+      </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>贷前尽调</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>面向客户经理和授信审查人员，围绕贷前尽调场景整合企业基本信息、经营现场、财务报表、流水税票、征信、司法舆情、关联方和担保圈等信息，自动生成尽调分析报告草稿、风险问题清单、补充材料清单和授信建议。</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="inlineStr">
+        <is>
+          <t>混合型 Skill（数据核验+规则+LLM报告生成+人工复核）</t>
+        </is>
+      </c>
+      <c r="J22" s="24" t="inlineStr">
+        <is>
+          <t>信贷</t>
+        </is>
+      </c>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>主 Skill + L1</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>混合型</t>
+        </is>
+      </c>
+      <c r="M22" s="24" t="inlineStr">
+        <is>
+          <t>仅Demo</t>
+        </is>
+      </c>
+      <c r="N22" s="24" t="inlineStr">
+        <is>
+          <t>企业工商信息、授信申请、财务报表、银行流水、税票、征信报告、司法舆情、合同/发票/年报/章程、现场走访记录、关联方与担保信息</t>
+        </is>
+      </c>
+      <c r="O22" s="24" t="inlineStr">
+        <is>
+          <t>信贷尽调分析报告草稿、风险评级/关注等级、风险问题清单、待补充材料清单、授信额度/期限/担保条件建议、后续跟踪要求</t>
+        </is>
+      </c>
+      <c r="P22" s="24" t="inlineStr">
+        <is>
+          <t>已制作</t>
+        </is>
+      </c>
+      <c r="Q22" s="24" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="R22" s="24" t="inlineStr">
+        <is>
+          <t>FDE共创/模拟Demo</t>
+        </is>
+      </c>
+      <c r="S22" s="24" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="T22" s="24" t="inlineStr">
+        <is>
+          <t>当前为售前演示 Demo，未伪造真实 SKILL.md；后续拿到真实业务规则、数据接口和脚本后，可补齐 Skill 包并升级为真实Skill包+Demo。</t>
+        </is>
+      </c>
+      <c r="U22" s="24" t="str"/>
+      <c r="V22" s="24" t="inlineStr">
+        <is>
+          <t>presales-skill-matrix/credit-due-diligence-report/credit-due-diligence-report-demo.html</t>
+        </is>
+      </c>
+      <c r="W22" s="24" t="str"/>
+      <c r="X22" s="24" t="str"/>
+      <c r="Y22" s="24" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="Z22" s="24" t="inlineStr">
+        <is>
+          <t>AI信贷,信贷,风控,贷前,尽调,尽调报告,授信审批,企业信用分析,财务分析,征信核查,关联担保,报告生成,仅Demo</t>
+        </is>
+      </c>
+      <c r="AA22" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-09 新增信贷尽调调查场景；Demo 使用脱敏模拟数据展示左侧业务工作台、中间 Skill 链路、右侧模拟数据区。</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="n"/>
@@ -11266,7 +11368,6 @@
       <c r="AA220" s="24" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA220"/>
   <dataValidations count="15">
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"客户金融场景,SA-AI内化场景"</formula1>

</xml_diff>